<commit_message>
Final version: Added Instructions tab to CAS Calculator
</commit_message>
<xml_diff>
--- a/CAS_Calculator.xlsx
+++ b/CAS_Calculator.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LENOVO\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{749685B4-897B-4B97-82BB-A020055422F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A97BCA8-0B64-4497-AF64-86DB4FB59019}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="732" yWindow="732" windowWidth="17280" windowHeight="8880" xr2:uid="{E4941081-D559-4FA0-8A85-AC04B9F77FF8}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{E4941081-D559-4FA0-8A85-AC04B9F77FF8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Variant ID</t>
   </si>
@@ -58,13 +59,206 @@
   </si>
   <si>
     <t>Suggested Modality</t>
+  </si>
+  <si>
+    <t>CRISPR Actionability Score (CAS) Calculator</t>
+  </si>
+  <si>
+    <r>
+      <t>Overview</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> This tool is designed to prioritize genome-wide significant Type 2 Diabetes (T2D) loci for functional interrogation based on the CAS framework.</t>
+    </r>
+  </si>
+  <si>
+    <t>How to Use This Tool:</t>
+  </si>
+  <si>
+    <r>
+      <t>Input Data</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">: Enter your variant information in the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>"Calculator"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> tab starting from Row 2.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>2. Assign Sub-Scores</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>: Input values for the four biological components:</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Genomic Context (0–3)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>: 3 for coding, 2 for non-coding with enhancer overlap, 1 for distal .</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Regulatory Evidence (0–3)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>: 3 for strong islet-specific enhancer overlap, 2 for moderate, 1 for limited .</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Expression Score (0–2)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>: 2 for High (TPM &gt;10), 1 for Moderate (TPM 1–10), 0 for Low (&lt;1) .</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Target Clarity (0–2)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>: 2 for a single effector, 1 for multiple candidates, 0 for ambiguous .</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>3. Review Results</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>: The sheet will automatically calculate:</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Total CAS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>: Maximum of 10.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Priority Tier</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>: High (≥7), Moderate (5–6), or Lower (&lt;5) .</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Suggested Modality</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>: CRISPR Knockout for coding vs. CRISPRi for non-coding regulatory .</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Note on Modality Assignment:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Assignments are strictly architecture-aligned to ensure experimental perturbation logic reflects variant biology.</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -79,6 +273,26 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13.5"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -101,13 +315,34 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -474,4 +709,126 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{68893547-E439-490B-95E4-50AE3E56CA41}">
+  <dimension ref="A1:A31"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:1" ht="17.399999999999999" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" s="5"/>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" s="5"/>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A10" s="5"/>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A11" s="7"/>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A12" s="8"/>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A13" s="9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A14" s="8"/>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A15" s="9" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A16" s="8"/>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A17" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A18" s="8"/>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A19" s="9" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A20" s="5"/>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A21" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A22" s="5"/>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A23" s="7"/>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A24" s="8"/>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A25" s="9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A26" s="8"/>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A27" s="9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A28" s="8"/>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A29" s="9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A31" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>